<commit_message>
Enhance block-design evaluation and export
Add comprehensive evaluation and export utilities for AlgDesign blocked designs: fix openxlsx worksheet dimension refs, add combine_blocked_design, evaluate_algdesign_block_design, and helpers to label, summarise and extract confounding/efficiency metrics. Introduce evaluate_block_summary and printing helpers to produce human-friendly summaries (D-score, condition number, within-block efficiencies, confounding summaries) and rename save_blocked_sets_to_excel parameter to `evaluation`. Update script to build a single optBlock for the chosen block size, run the new evaluations, save results to vignette_sets.xlsx, and perform workbook integrity checks. Updated generated XLSX outputs accordingly.
</commit_message>
<xml_diff>
--- a/outputs/vignette_sets.xlsx
+++ b/outputs/vignette_sets.xlsx
@@ -36,7 +36,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+  <si>
+    <t xml:space="preserve">candidate_design</t>
+  </si>
   <si>
     <t xml:space="preserve">set_size</t>
   </si>
@@ -47,16 +50,82 @@
     <t xml:space="preserve">n_vignettes</t>
   </si>
   <si>
-    <t xml:space="preserve">determinant_efficiency</t>
+    <t xml:space="preserve">model_terms</t>
   </si>
   <si>
-    <t xml:space="preserve">trace_efficiency</t>
+    <t xml:space="preserve">n_parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">design_matrix_rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameters_estimable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">full_rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">condition_number_lower_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_score_higher_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">optblock_d_higher_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">optblock_diagonality_higher_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">centered_within_term_determinant_higher_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">within_block_efficiency_det_higher_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">within_block_efficiency_trace_higher_is_better</t>
   </si>
   <si>
     <t xml:space="preserve">rho</t>
   </si>
   <si>
-    <t xml:space="preserve">max_abs_confounding</t>
+    <t xml:space="preserve">max_abs_confounding_offdiag_lower_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">strongest_confounding_terms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_abs_confounding_ge_0_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_abs_confounding_ge_0_25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_abs_cross_factor_confounding_lower_is_better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">strongest_cross_factor_confounding_terms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_abs_cross_factor_confounding_ge_0_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_abs_cross_factor_confounding_ge_0_25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 respondent sets x 4 vignettes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A + B + C + D + E + F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8/8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3 with C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">none</t>
   </si>
   <si>
     <t xml:space="preserve">A</t>
@@ -422,16 +491,34 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="designevaluation" displayName="designevaluation" ref="A1:G2" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:G2"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="set_size"/>
-    <tableColumn id="2" name="n_sets"/>
-    <tableColumn id="3" name="n_vignettes"/>
-    <tableColumn id="4" name="determinant_efficiency"/>
-    <tableColumn id="5" name="trace_efficiency"/>
-    <tableColumn id="6" name="rho"/>
-    <tableColumn id="7" name="max_abs_confounding"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="designevaluation" displayName="designevaluation" ref="A1:Y2" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:Y2"/>
+  <tableColumns count="25">
+    <tableColumn id="1" name="candidate_design"/>
+    <tableColumn id="2" name="set_size"/>
+    <tableColumn id="3" name="n_sets"/>
+    <tableColumn id="4" name="n_vignettes"/>
+    <tableColumn id="5" name="model_terms"/>
+    <tableColumn id="6" name="n_parameters"/>
+    <tableColumn id="7" name="design_matrix_rank"/>
+    <tableColumn id="8" name="parameters_estimable"/>
+    <tableColumn id="9" name="full_rank"/>
+    <tableColumn id="10" name="condition_number_lower_is_better"/>
+    <tableColumn id="11" name="d_score_higher_is_better"/>
+    <tableColumn id="12" name="optblock_d_higher_is_better"/>
+    <tableColumn id="13" name="optblock_diagonality_higher_is_better"/>
+    <tableColumn id="14" name="centered_within_term_determinant_higher_is_better"/>
+    <tableColumn id="15" name="within_block_efficiency_det_higher_is_better"/>
+    <tableColumn id="16" name="within_block_efficiency_trace_higher_is_better"/>
+    <tableColumn id="17" name="rho"/>
+    <tableColumn id="18" name="max_abs_confounding_offdiag_lower_is_better"/>
+    <tableColumn id="19" name="strongest_confounding_terms"/>
+    <tableColumn id="20" name="n_abs_confounding_ge_0_10"/>
+    <tableColumn id="21" name="n_abs_confounding_ge_0_25"/>
+    <tableColumn id="22" name="max_abs_cross_factor_confounding_lower_is_better"/>
+    <tableColumn id="23" name="strongest_cross_factor_confounding_terms"/>
+    <tableColumn id="24" name="n_abs_cross_factor_confounding_ge_0_10"/>
+    <tableColumn id="25" name="n_abs_cross_factor_confounding_ge_0_25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -812,16 +899,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="8.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="6.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="5.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="19.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="32.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="8.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="6.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="21.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="12.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="18.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="20.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="9.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="32.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="24.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="27.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="37.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="49.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="44.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="46.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="3.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="43.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="27.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="25.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="25.71" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="48.71" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="40.71" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="38.71" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="38.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -846,28 +951,136 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" t="n">
         <v>4</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>24</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>96</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
+      <c r="J2" t="n">
+        <v>36.0647646382379</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.278478733344532</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.227071279701159</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.278478733344532</v>
+      </c>
+      <c r="O2" t="n">
         <v>0.983</v>
       </c>
-      <c r="F2" t="n">
+      <c r="P2" t="n">
         <v>0.979</v>
       </c>
-      <c r="G2" t="n">
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="n">
         <v>0.5</v>
+      </c>
+      <c r="S2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U2" t="n">
+        <v>2</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="s">
+        <v>29</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -881,7 +1094,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -895,45 +1108,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>4</v>
@@ -941,22 +1154,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>17</v>
@@ -964,22 +1177,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>78</v>
@@ -987,22 +1200,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>95</v>
@@ -1019,7 +1232,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1033,45 +1246,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>18</v>
@@ -1079,22 +1292,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>27</v>
@@ -1102,22 +1315,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>69</v>
@@ -1125,22 +1338,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>84</v>
@@ -1157,7 +1370,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1171,45 +1384,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>14</v>
@@ -1217,22 +1430,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>31</v>
@@ -1240,22 +1453,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>63</v>
@@ -1263,22 +1476,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>82</v>
@@ -1295,7 +1508,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1309,45 +1522,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>19</v>
@@ -1355,22 +1568,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>22</v>
@@ -1378,22 +1591,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>73</v>
@@ -1401,22 +1614,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>80</v>
@@ -1433,7 +1646,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1447,45 +1660,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>6</v>
@@ -1493,22 +1706,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>16</v>
@@ -1516,22 +1729,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>83</v>
@@ -1539,22 +1752,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>89</v>
@@ -1571,7 +1784,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1585,45 +1798,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>2</v>
@@ -1631,22 +1844,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>23</v>
@@ -1654,22 +1867,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>56</v>
@@ -1677,22 +1890,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>93</v>
@@ -1709,7 +1922,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1723,45 +1936,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>35</v>
@@ -1769,22 +1982,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>43</v>
@@ -1792,22 +2005,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>70</v>
@@ -1815,22 +2028,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>74</v>
@@ -1847,7 +2060,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1861,45 +2074,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>28</v>
@@ -1907,22 +2120,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>48</v>
@@ -1930,22 +2143,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>49</v>
@@ -1953,22 +2166,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>65</v>
@@ -1985,7 +2198,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -1999,45 +2212,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>11</v>
@@ -2045,22 +2258,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>38</v>
@@ -2068,22 +2281,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>54</v>
@@ -2091,22 +2304,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>91</v>
@@ -2123,7 +2336,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -2137,45 +2350,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>10</v>
@@ -2183,22 +2396,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>39</v>
@@ -2206,22 +2419,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>51</v>
@@ -2229,22 +2442,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>90</v>
@@ -2261,7 +2474,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -2275,45 +2488,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>26</v>
@@ -2321,22 +2534,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>47</v>
@@ -2344,22 +2557,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>53</v>
@@ -2367,22 +2580,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>64</v>
@@ -2399,7 +2612,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -2413,45 +2626,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>5</v>
@@ -2459,22 +2672,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>41</v>
@@ -2482,22 +2695,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>52</v>
@@ -2505,22 +2718,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>96</v>
@@ -2537,7 +2750,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -2551,45 +2764,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>7</v>
@@ -2597,22 +2810,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>44</v>
@@ -2620,22 +2833,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>62</v>
@@ -2643,22 +2856,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>81</v>
@@ -2675,7 +2888,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -2689,45 +2902,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>29</v>
@@ -2735,22 +2948,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>37</v>
@@ -2758,22 +2971,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>60</v>
@@ -2781,22 +2994,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>72</v>
@@ -2813,7 +3026,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -2827,45 +3040,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>20</v>
@@ -2873,22 +3086,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>36</v>
@@ -2896,22 +3109,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>57</v>
@@ -2919,22 +3132,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>85</v>
@@ -2951,7 +3164,7 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -2965,45 +3178,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>12</v>
@@ -3011,22 +3224,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>33</v>
@@ -3034,22 +3247,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>61</v>
@@ -3057,22 +3270,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>92</v>
@@ -3089,7 +3302,7 @@
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -3103,45 +3316,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>24</v>
@@ -3149,22 +3362,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>25</v>
@@ -3172,22 +3385,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>68</v>
@@ -3195,22 +3408,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>77</v>
@@ -3227,7 +3440,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -3241,45 +3454,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>15</v>
@@ -3287,22 +3500,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>34</v>
@@ -3310,22 +3523,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>66</v>
@@ -3333,22 +3546,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>75</v>
@@ -3365,7 +3578,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -3379,45 +3592,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>9</v>
@@ -3425,22 +3638,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>42</v>
@@ -3448,22 +3661,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>59</v>
@@ -3471,22 +3684,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>88</v>
@@ -3503,7 +3716,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -3517,45 +3730,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>32</v>
@@ -3563,22 +3776,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>45</v>
@@ -3586,22 +3799,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>50</v>
@@ -3609,22 +3822,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>67</v>
@@ -3641,7 +3854,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -3655,45 +3868,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -3701,22 +3914,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>8</v>
@@ -3724,22 +3937,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>87</v>
@@ -3747,22 +3960,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>94</v>
@@ -3779,7 +3992,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -3793,45 +4006,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>13</v>
@@ -3839,22 +4052,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>40</v>
@@ -3862,22 +4075,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>58</v>
@@ -3885,22 +4098,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>79</v>
@@ -3917,7 +4130,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -3931,45 +4144,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>3</v>
@@ -3977,22 +4190,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>30</v>
@@ -4000,22 +4213,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>71</v>
@@ -4023,22 +4236,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>86</v>
@@ -4055,7 +4268,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="3.71" hidden="0" customWidth="1"/>
@@ -4069,45 +4282,45 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G2" t="n">
         <v>21</v>
@@ -4115,22 +4328,22 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
         <v>46</v>
@@ -4138,22 +4351,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G4" t="n">
         <v>55</v>
@@ -4161,22 +4374,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
         <v>76</v>

</xml_diff>